<commit_message>
Make daily earnings runner resilient per symbol
</commit_message>
<xml_diff>
--- a/exports/daily_trades_2026-07-15.xlsx
+++ b/exports/daily_trades_2026-07-15.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,6 +478,744 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ABT</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>87.94000244140625</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Iron Condor</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>38</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-6.186038538071315</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-11.87173317212761</v>
+      </c>
+      <c r="G2" t="n">
+        <v>6.891059120258136</v>
+      </c>
+      <c r="H2" t="n">
+        <v>12.57675375431442</v>
+      </c>
+      <c r="I2" t="n">
+        <v>82.5</v>
+      </c>
+      <c r="J2" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="K2" t="n">
+        <v>94</v>
+      </c>
+      <c r="L2" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CBSH</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>57.81999969482422</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Iron Condor</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>28</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-13.52473147024978</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-22.1722583232248</v>
+      </c>
+      <c r="G3" t="n">
+        <v>12.41784908867529</v>
+      </c>
+      <c r="H3" t="n">
+        <v>21.0653759416503</v>
+      </c>
+      <c r="I3" t="n">
+        <v>50</v>
+      </c>
+      <c r="J3" t="n">
+        <v>45</v>
+      </c>
+      <c r="K3" t="n">
+        <v>65</v>
+      </c>
+      <c r="L3" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CFG</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>70.69000244140625</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Iron Condor</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>38</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-8.049232203836176</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-15.12236818815646</v>
+      </c>
+      <c r="G4" t="n">
+        <v>6.097039764804424</v>
+      </c>
+      <c r="H4" t="n">
+        <v>13.17017574912471</v>
+      </c>
+      <c r="I4" t="n">
+        <v>65</v>
+      </c>
+      <c r="J4" t="n">
+        <v>60</v>
+      </c>
+      <c r="K4" t="n">
+        <v>75</v>
+      </c>
+      <c r="L4" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>FEIM</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>59.00400161743164</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Iron Condor</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>28</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-15.25998469698973</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-23.73398622729076</v>
+      </c>
+      <c r="G5" t="n">
+        <v>18.63602142421439</v>
+      </c>
+      <c r="H5" t="n">
+        <v>27.11002295451541</v>
+      </c>
+      <c r="I5" t="n">
+        <v>50</v>
+      </c>
+      <c r="J5" t="n">
+        <v>45</v>
+      </c>
+      <c r="K5" t="n">
+        <v>70</v>
+      </c>
+      <c r="L5" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>GE</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>355.6400146484375</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Iron Condor</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>38</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-5.80362551971011</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-11.42728966778712</v>
+      </c>
+      <c r="G6" t="n">
+        <v>6.849618813463154</v>
+      </c>
+      <c r="H6" t="n">
+        <v>12.47328296154016</v>
+      </c>
+      <c r="I6" t="n">
+        <v>335</v>
+      </c>
+      <c r="J6" t="n">
+        <v>315</v>
+      </c>
+      <c r="K6" t="n">
+        <v>380</v>
+      </c>
+      <c r="L6" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>GSBC</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>77.44000244140625</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Iron Condor</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>28</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-9.607440866283046</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-16.06405223297711</v>
+      </c>
+      <c r="G7" t="n">
+        <v>9.762393233799171</v>
+      </c>
+      <c r="H7" t="n">
+        <v>16.21900460049324</v>
+      </c>
+      <c r="I7" t="n">
+        <v>70</v>
+      </c>
+      <c r="J7" t="n">
+        <v>65</v>
+      </c>
+      <c r="K7" t="n">
+        <v>85</v>
+      </c>
+      <c r="L7" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>HOMB</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>29.14999961853027</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Short Strangle</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>28</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-14.23670556720067</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-22.8130350104806</v>
+      </c>
+      <c r="G8" t="n">
+        <v>20.06861220591907</v>
+      </c>
+      <c r="I8" t="n">
+        <v>25</v>
+      </c>
+      <c r="J8" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="K8" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>IIIN</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>29.73999977111816</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Iron Condor</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>28</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-15.93812981707346</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-24.34431683536612</v>
+      </c>
+      <c r="G9" t="n">
+        <v>17.68661825609714</v>
+      </c>
+      <c r="H9" t="n">
+        <v>31.13651748536539</v>
+      </c>
+      <c r="I9" t="n">
+        <v>25</v>
+      </c>
+      <c r="J9" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="K9" t="n">
+        <v>35</v>
+      </c>
+      <c r="L9" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>JBHT</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>278.8200073242188</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Iron Condor</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>28</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-10.33642011590156</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-13.9229633112655</v>
+      </c>
+      <c r="G10" t="n">
+        <v>7.596295860918123</v>
+      </c>
+      <c r="H10" t="n">
+        <v>11.18283905628206</v>
+      </c>
+      <c r="I10" t="n">
+        <v>250</v>
+      </c>
+      <c r="J10" t="n">
+        <v>240</v>
+      </c>
+      <c r="K10" t="n">
+        <v>300</v>
+      </c>
+      <c r="L10" t="n">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>MAN</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>39.68989944458008</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Short Strangle</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>28</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-24.41401862987914</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-37.01168219156595</v>
+      </c>
+      <c r="G11" t="n">
+        <v>13.37897205518128</v>
+      </c>
+      <c r="I11" t="n">
+        <v>30</v>
+      </c>
+      <c r="J11" t="n">
+        <v>25</v>
+      </c>
+      <c r="K11" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>PLD</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>143.0549926757812</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Iron Condor</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>28</v>
+      </c>
+      <c r="E12" t="n">
+        <v>-5.630696646874133</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-9.125856030323243</v>
+      </c>
+      <c r="G12" t="n">
+        <v>4.854781503473182</v>
+      </c>
+      <c r="H12" t="n">
+        <v>8.34994088692229</v>
+      </c>
+      <c r="I12" t="n">
+        <v>135</v>
+      </c>
+      <c r="J12" t="n">
+        <v>130</v>
+      </c>
+      <c r="K12" t="n">
+        <v>150</v>
+      </c>
+      <c r="L12" t="n">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>185.0749969482422</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Iron Condor</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>28</v>
+      </c>
+      <c r="E13" t="n">
+        <v>-5.443737465552811</v>
+      </c>
+      <c r="F13" t="n">
+        <v>-10.84695246752122</v>
+      </c>
+      <c r="G13" t="n">
+        <v>8.064300039368222</v>
+      </c>
+      <c r="H13" t="n">
+        <v>13.46751504133663</v>
+      </c>
+      <c r="I13" t="n">
+        <v>175</v>
+      </c>
+      <c r="J13" t="n">
+        <v>165</v>
+      </c>
+      <c r="K13" t="n">
+        <v>200</v>
+      </c>
+      <c r="L13" t="n">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TRX</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.8179000020027161</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Short Strangle</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>28</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-38.86783240302039</v>
+      </c>
+      <c r="G14" t="n">
+        <v>83.39650279093884</v>
+      </c>
+      <c r="H14" t="n">
+        <v>511.3216759697961</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K14" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="L14" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>TSM</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>423.864990234375</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Iron Condor</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>48</v>
+      </c>
+      <c r="E15" t="n">
+        <v>-5.630328237578408</v>
+      </c>
+      <c r="F15" t="n">
+        <v>-10.34881182569949</v>
+      </c>
+      <c r="G15" t="n">
+        <v>6.165880732724283</v>
+      </c>
+      <c r="H15" t="n">
+        <v>10.88436432084536</v>
+      </c>
+      <c r="I15" t="n">
+        <v>400</v>
+      </c>
+      <c r="J15" t="n">
+        <v>380</v>
+      </c>
+      <c r="K15" t="n">
+        <v>450</v>
+      </c>
+      <c r="L15" t="n">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>UAL</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>120.9899978637695</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Iron Condor</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>38</v>
+      </c>
+      <c r="E16" t="n">
+        <v>-6.603849908953618</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-10.73642292183178</v>
+      </c>
+      <c r="G16" t="n">
+        <v>7.446898334832119</v>
+      </c>
+      <c r="H16" t="n">
+        <v>11.57947134771027</v>
+      </c>
+      <c r="I16" t="n">
+        <v>113</v>
+      </c>
+      <c r="J16" t="n">
+        <v>108</v>
+      </c>
+      <c r="K16" t="n">
+        <v>130</v>
+      </c>
+      <c r="L16" t="n">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>417.25</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Iron Condor</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>48</v>
+      </c>
+      <c r="E17" t="n">
+        <v>-6.530856800479334</v>
+      </c>
+      <c r="F17" t="n">
+        <v>-11.32414619532654</v>
+      </c>
+      <c r="G17" t="n">
+        <v>6.65068903535051</v>
+      </c>
+      <c r="H17" t="n">
+        <v>11.44397843019773</v>
+      </c>
+      <c r="I17" t="n">
+        <v>390</v>
+      </c>
+      <c r="J17" t="n">
+        <v>370</v>
+      </c>
+      <c r="K17" t="n">
+        <v>445</v>
+      </c>
+      <c r="L17" t="n">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>USB</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>62.45999908447266</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Iron Condor</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>48</v>
+      </c>
+      <c r="E18" t="n">
+        <v>-3.938519245166305</v>
+      </c>
+      <c r="F18" t="n">
+        <v>-11.94364264140245</v>
+      </c>
+      <c r="G18" t="n">
+        <v>4.06660415106983</v>
+      </c>
+      <c r="H18" t="n">
+        <v>12.07172754730597</v>
+      </c>
+      <c r="I18" t="n">
+        <v>60</v>
+      </c>
+      <c r="J18" t="n">
+        <v>55</v>
+      </c>
+      <c r="K18" t="n">
+        <v>65</v>
+      </c>
+      <c r="L18" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>WIT</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1.850000023841858</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Iron Condor</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>28</v>
+      </c>
+      <c r="E19" t="n">
+        <v>-45.94594664256706</v>
+      </c>
+      <c r="F19" t="n">
+        <v>-72.97297332128353</v>
+      </c>
+      <c r="G19" t="n">
+        <v>170.2702667871647</v>
+      </c>
+      <c r="H19" t="n">
+        <v>305.4054001807471</v>
+      </c>
+      <c r="I19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K19" t="n">
+        <v>5</v>
+      </c>
+      <c r="L19" t="n">
+        <v>7.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>